<commit_message>
update factor 2 and 3
</commit_message>
<xml_diff>
--- a/Data/Bronze/MCIC-PROFUNDIZACION/Procesos de Renocavion y acreditación/Plan de Mejoramiento/FACTOR 3. PROFESORES/a. Informes de participación de los docentes/F3_Participacion_Docente_Capacitacion.xlsx
+++ b/Data/Bronze/MCIC-PROFUNDIZACION/Procesos de Renocavion y acreditación/Plan de Mejoramiento/FACTOR 3. PROFESORES/a. Informes de participación de los docentes/F3_Participacion_Docente_Capacitacion.xlsx
@@ -9,11 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacitación docente" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movilidad" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certificados" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movilidad" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Capacitación docente'!$A$4:$J$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Movilidad'!$A$4:$I$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Capacitación docente'!$A$4:$J$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Certificados'!$A$4:$G$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Movilidad'!$A$4:$I$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -599,10 +601,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Participación de los profesores de la Maestría en capacitación académica y administrativa, y movilidad académica. Información en actualización: se solicitó a los profesores reportar con soporte las capacitaciones adicionales del periodo 2025-2026 (columna J de la hoja «Capacitación docente»).</t>
+          <t>Participación de los profesores de la Maestría en capacitación académica y administrativa, y movilidad académica. Incluye las capacitaciones adicionales con certificado reportadas por los profesores (columna J de la hoja «Capacitación docente» y hoja «Certificados»).</t>
         </is>
       </c>
     </row>
@@ -691,14 +693,14 @@
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>43 %</t>
+          <t>48 %</t>
         </is>
       </c>
       <c r="G10" s="9" t="n">
@@ -743,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -755,7 +757,7 @@
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -820,7 +822,7 @@
       </c>
       <c r="J4" s="11" t="inlineStr">
         <is>
-          <t>Capacitaciones 2025-2026 reportadas por el profesor (por diligenciar)</t>
+          <t>Otras capacitaciones con certificado</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1256,11 @@
           <t>Asociado</t>
         </is>
       </c>
-      <c r="J20" s="12" t="n"/>
+      <c r="J20" s="12" t="inlineStr">
+        <is>
+          <t>Taller de formación EUR-ACE «Aseguramiento de calidad y acreditación internacional EUR-ACE de programas educativos en ingeniería» — ENAEE, ENTEA y LACCEI (Girardot, Colombia) (08/11/2022 al 10/11/2022)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
@@ -1394,7 +1400,12 @@
           <t>Asociado</t>
         </is>
       </c>
-      <c r="J25" s="6" t="n"/>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>Introduction to GeoWebApp Building with open-source tools (curso en línea) — Universidad de Twente (ITC) y Geoversity (13/05/2024, 40 h)
+Curso Internacional de Competencias Docentes y Diseño de Materiales Didácticos para la Educación en Línea (título propio, calificación 9,60) — Universidad Internacional de La Rioja (UNIR) (04/05/2026 al 05/07/2026, 125 h)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="n">
@@ -1458,7 +1469,11 @@
       </c>
       <c r="H27" s="6" t="n"/>
       <c r="I27" s="6" t="n"/>
-      <c r="J27" s="6" t="n"/>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>Data Science and Machine Learning: Making Data-Driven Decisions — MIT Schwarzman College of Computing y MIT IDSS (agosto de 2023)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="n">
@@ -1628,30 +1643,54 @@
       </c>
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>Vera Parra Nelson Enrique</t>
-        </is>
-      </c>
-      <c r="C34" s="12" t="inlineStr">
-        <is>
-          <t>Titular</t>
-        </is>
-      </c>
+          <t>Vanegas Ayala Sebastian Camilo</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="n"/>
       <c r="D34" s="12" t="n"/>
       <c r="E34" s="12" t="n"/>
-      <c r="F34" s="12" t="inlineStr">
-        <is>
-          <t>Curso y aprobo especializado I y II 2023-1</t>
-        </is>
-      </c>
-      <c r="G34" s="12" t="n">
-        <v>2023</v>
-      </c>
+      <c r="F34" s="12" t="n"/>
+      <c r="G34" s="12" t="n"/>
       <c r="H34" s="12" t="n"/>
       <c r="I34" s="12" t="n"/>
-      <c r="J34" s="12" t="n"/>
+      <c r="J34" s="12" t="inlineStr">
+        <is>
+          <t>Taller «Instalación local de modelos de IA» — Vicerrectoría Académica y Comité PlanEsTIC-UD (16/07/2025, 1 h)
+Taller «Automatización de tareas de ofimática con IA a través del uso de protocolo MCP» — Vicerrectoría Académica y Comité PlanEsTIC-UD (15/07/2025, 1 h)
+Taller «Da vida a tus ideas con presentaciones creativas e impactantes en Gamma AI» — Vicerrectoría Académica y Comité PlanEsTIC-UD (20/08/2025, 1 h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Vera Parra Nelson Enrique</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Titular</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Curso y aprobo especializado I y II 2023-1</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H35" s="6" t="n"/>
+      <c r="I35" s="6" t="n"/>
+      <c r="J35" s="6" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J34"/>
+  <autoFilter ref="A4:J35"/>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
@@ -1661,6 +1700,320 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Capacitaciones con certificado reportadas por los profesores</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Certificados recientes entregados por los profesores; los documentos se resguardan en el archivo del programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Profesor</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Capacitación</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Entidad</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Horas</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Año</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Soporte</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Gomez Vargas Ernesto</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Taller de formación EUR-ACE «Aseguramiento de calidad y acreditación internacional EUR-ACE de programas educativos en ingeniería»</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>ENAEE, ENTEA y LACCEI (Girardot, Colombia)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>08/11/2022 al 10/11/2022</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>2022</v>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Certificado en archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Ortiz Davila Alvaro Enrique</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Introduction to GeoWebApp Building with open-source tools (curso en línea)</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Universidad de Twente (ITC) y Geoversity</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>13/05/2024</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>2024</v>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>Certificado en archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Ortiz Davila Alvaro Enrique</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Curso Internacional de Competencias Docentes y Diseño de Materiales Didácticos para la Educación en Línea (título propio, calificación 9,60)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Universidad Internacional de La Rioja (UNIR)</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>04/05/2026 al 05/07/2026</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>125</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Certificado en archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Plazas Nossa Leonardo</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Data Science and Machine Learning: Making Data-Driven Decisions</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>MIT Schwarzman College of Computing y MIT IDSS</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>agosto de 2023</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>Certificado en archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Vanegas Ayala Sebastian Camilo</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Taller «Instalación local de modelos de IA»</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Vicerrectoría Académica y Comité PlanEsTIC-UD</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>16/07/2025</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Certificado en archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Vanegas Ayala Sebastian Camilo</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Taller «Automatización de tareas de ofimática con IA a través del uso de protocolo MCP»</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Vicerrectoría Académica y Comité PlanEsTIC-UD</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>15/07/2025</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="12" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>Certificado en archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Vanegas Ayala Sebastian Camilo</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Taller «Da vida a tus ideas con presentaciones creativas e impactantes en Gamma AI»</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Vicerrectoría Académica y Comité PlanEsTIC-UD</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>20/08/2025</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Certificado en archivo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G11"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>